<commit_message>
docs(hw03): align checklist data with seeded SUT
</commit_message>
<xml_diff>
--- a/hw03/submission/23127065/23127065_HW03_GUI_Checklist.xlsx
+++ b/hw03/submission/23127065/23127065_HW03_GUI_Checklist.xlsx
@@ -266,7 +266,7 @@
     <t>IA-01, IA-02, IA-04</t>
   </si>
   <si>
-    <t>Thêm Sản phẩm A và B rồi mở `/cart`.</t>
+    <t>Thêm iPhone 15 Pro Max và Samsung Galaxy S24 Ultra rồi mở `/cart`.</t>
   </si>
   <si>
     <t>Mỗi sản phẩm xuất hiện đúng một dòng và đúng thứ tự hiển thị dự kiến.</t>
@@ -368,10 +368,10 @@
     <t>CART-GUI-021</t>
   </si>
   <si>
-    <t>Thêm cùng Sản phẩm A lần lượt với số lượng 1 và 2.</t>
-  </si>
-  <si>
-    <t>Chỉ có một dòng Sản phẩm A với số lượng 3; không tạo hai dòng trùng lặp.</t>
+    <t>Thêm cùng iPhone 15 Pro Max lần lượt với số lượng 1 và 2.</t>
+  </si>
+  <si>
+    <t>Chỉ có một dòng iPhone 15 Pro Max với số lượng 3; không tạo hai dòng trùng lặp.</t>
   </si>
   <si>
     <t>BUG-CART-12</t>

</xml_diff>